<commit_message>
added omnium individual race rankings based off overall rankings
</commit_message>
<xml_diff>
--- a/pages/WR_progressions/Mens_Progression.xlsx
+++ b/pages/WR_progressions/Mens_Progression.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/anja_kuys_hpsnz_org_nz/Documents/Desktop/Scripts/CNZPD/pages/WR_progressions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_FF6BE833DD9E4E317729F09F5470CA66DBC2C15B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_FF6BE833DD9E4E317729F09F5470CA66DBC2C15B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58490DAC-1E65-4B53-9254-F8071515AB94}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1620" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Medals_F200" sheetId="1" r:id="rId1"/>
@@ -18,8 +18,8 @@
     <sheet name="Medals_TP" sheetId="3" r:id="rId3"/>
     <sheet name="Medals_TS" sheetId="4" r:id="rId4"/>
     <sheet name="Medals_Madison" sheetId="5" r:id="rId5"/>
-    <sheet name="Medals_Om_Scratch" sheetId="6" r:id="rId6"/>
-    <sheet name="Medals_Om_Tempo" sheetId="7" r:id="rId7"/>
+    <sheet name="Medals_Om_Tempo" sheetId="7" r:id="rId6"/>
+    <sheet name="Medals_Om_Scratch" sheetId="6" r:id="rId7"/>
     <sheet name="Medals_Om_Elim" sheetId="8" r:id="rId8"/>
     <sheet name="Medals_Om_Points" sheetId="9" r:id="rId9"/>
     <sheet name="WR_F200" sheetId="10" r:id="rId10"/>
@@ -32,9 +32,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Medals_IP!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Medals_Madison!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Medals_Om_Elim!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Medals_Om_Points!$A$1:$R$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Medals_Om_Scratch!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Medals_Om_Tempo!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Medals_Om_Points!$A$1:$R$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Medals_Om_Scratch!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Medals_Om_Tempo!$A$1:$L$133</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Medals_TP!$A$1:$Y$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Medals_TS!$A$1:$H$1</definedName>
   </definedNames>
@@ -20288,1164 +20288,8 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:H45"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.1796875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>177</v>
-      </c>
-      <c r="F1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G1" t="s">
-        <v>178</v>
-      </c>
-      <c r="H1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="9">
-        <v>2026</v>
-      </c>
-      <c r="C2" s="10">
-        <v>46136</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="G2" s="9">
-        <v>25.62191780821918</v>
-      </c>
-      <c r="H2" s="9">
-        <v>55.640999999999998</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="11">
-        <v>2026</v>
-      </c>
-      <c r="C3" s="12">
-        <v>46129</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="G3" s="11">
-        <v>23.55890410958904</v>
-      </c>
-      <c r="H3" s="11">
-        <v>56.962000000000003</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="9">
-        <v>2025</v>
-      </c>
-      <c r="C4" s="10">
-        <v>45952</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="G4" s="9">
-        <v>36.402739726027399</v>
-      </c>
-      <c r="H4" s="9">
-        <v>57.143000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B5" s="11">
-        <v>2025</v>
-      </c>
-      <c r="C5" s="12">
-        <v>45730</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="G5" s="11">
-        <v>23.80821917808219</v>
-      </c>
-      <c r="H5" s="11">
-        <v>54.381</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="9">
-        <v>2024</v>
-      </c>
-      <c r="C6" s="10">
-        <v>45584</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="G6" s="9">
-        <v>24.109589041095891</v>
-      </c>
-      <c r="H6" s="9">
-        <v>56.515000000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="11">
-        <v>2024</v>
-      </c>
-      <c r="C7" s="12">
-        <v>45512</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="G7" s="11">
-        <v>28.92602739726027</v>
-      </c>
-      <c r="H7" s="11">
-        <v>58.442</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="9">
-        <v>2024</v>
-      </c>
-      <c r="C8" s="10">
-        <v>45395</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="G8" s="9">
-        <v>37.536986301369858</v>
-      </c>
-      <c r="H8" s="9">
-        <v>56.25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="11">
-        <v>2024</v>
-      </c>
-      <c r="C9" s="12">
-        <v>45368</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="G9" s="11">
-        <v>21.473972602739721</v>
-      </c>
-      <c r="H9" s="11">
-        <v>55.728000000000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="9">
-        <v>2024</v>
-      </c>
-      <c r="C10" s="10">
-        <v>45325</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="G10" s="9">
-        <v>35.010958904109593</v>
-      </c>
-      <c r="H10" s="9">
-        <v>53.892000000000003</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="11">
-        <v>2023</v>
-      </c>
-      <c r="C11" s="12">
-        <v>45144</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="G11" s="11">
-        <v>25.109589041095891</v>
-      </c>
-      <c r="H11" s="11">
-        <v>54.795000000000002</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="9">
-        <v>2023</v>
-      </c>
-      <c r="C12" s="10">
-        <v>45038</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="G12" s="9">
-        <v>24.232876712328771</v>
-      </c>
-      <c r="H12" s="9">
-        <v>55.901000000000003</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="11">
-        <v>2023</v>
-      </c>
-      <c r="C13" s="12">
-        <v>45001</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="G13" s="11">
-        <v>29.07397260273973</v>
-      </c>
-      <c r="H13" s="11">
-        <v>53.097000000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="9">
-        <v>2023</v>
-      </c>
-      <c r="C14" s="10">
-        <v>44982</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="G14" s="9">
-        <v>27.761643835616439</v>
-      </c>
-      <c r="H14" s="9">
-        <v>52.173999999999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="11">
-        <v>2022</v>
-      </c>
-      <c r="C15" s="12">
-        <v>44849</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15" s="11">
-        <v>31.906849315068492</v>
-      </c>
-      <c r="H15" s="11"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" s="9">
-        <v>2022</v>
-      </c>
-      <c r="C16" s="10">
-        <v>44752</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="G16" s="9">
-        <v>28.465753424657539</v>
-      </c>
-      <c r="H16" s="9">
-        <v>52.631999999999998</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="11">
-        <v>2022</v>
-      </c>
-      <c r="C17" s="12">
-        <v>44696</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G17" s="11">
-        <v>23.671232876712331</v>
-      </c>
-      <c r="H17" s="11">
-        <v>53.097000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" s="9">
-        <v>2022</v>
-      </c>
-      <c r="C18" s="10">
-        <v>44675</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>183</v>
-      </c>
-      <c r="G18" s="9">
-        <v>26.42739726027397</v>
-      </c>
-      <c r="H18" s="9">
-        <v>54.545000000000002</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="11">
-        <v>2021</v>
-      </c>
-      <c r="C19" s="12">
-        <v>44492</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G19" s="11">
-        <v>23.112328767123291</v>
-      </c>
-      <c r="H19" s="11">
-        <v>55.47</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B20" s="9">
-        <v>2021</v>
-      </c>
-      <c r="C20" s="10">
-        <v>44451</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="G20" s="9">
-        <v>30.668493150684931</v>
-      </c>
-      <c r="H20" s="9">
-        <v>51.551000000000002</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="11">
-        <v>2021</v>
-      </c>
-      <c r="C21" s="12">
-        <v>44413</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G21" s="11">
-        <v>23.30958904109589</v>
-      </c>
-      <c r="H21" s="11">
-        <v>56.539000000000001</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" s="9">
-        <v>2021</v>
-      </c>
-      <c r="C22" s="10">
-        <v>44388</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="G22" s="9">
-        <v>23.038356164383561</v>
-      </c>
-      <c r="H22" s="9">
-        <v>53.85</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B23" s="11">
-        <v>2020</v>
-      </c>
-      <c r="C23" s="12">
-        <v>43890</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="F23" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="G23" s="11">
-        <v>24.482191780821921</v>
-      </c>
-      <c r="H23" s="11"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B24" s="9">
-        <v>2020</v>
-      </c>
-      <c r="C24" s="10">
-        <v>43855</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G24" s="9">
-        <v>25.164383561643831</v>
-      </c>
-      <c r="H24" s="9">
-        <v>53.784999999999997</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="11">
-        <v>2019</v>
-      </c>
-      <c r="C25" s="12">
-        <v>43813</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="F25" s="11" t="s">
-        <v>188</v>
-      </c>
-      <c r="G25" s="11">
-        <v>26.013698630136989</v>
-      </c>
-      <c r="H25" s="11">
-        <v>53.875</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B26" s="9">
-        <v>2019</v>
-      </c>
-      <c r="C26" s="10">
-        <v>43806</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G26" s="9">
-        <v>25.030136986301368</v>
-      </c>
-      <c r="H26" s="9">
-        <v>54.192999999999998</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B27" s="11">
-        <v>2019</v>
-      </c>
-      <c r="C27" s="12">
-        <v>43799</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="F27" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="G27" s="11">
-        <v>31.8</v>
-      </c>
-      <c r="H27" s="11">
-        <v>53.749000000000002</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A28" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B28" s="9">
-        <v>2019</v>
-      </c>
-      <c r="C28" s="10">
-        <v>43779</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="G28" s="9">
-        <v>23.82465753424658</v>
-      </c>
-      <c r="H28" s="9"/>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B29" s="11">
-        <v>2019</v>
-      </c>
-      <c r="C29" s="12">
-        <v>43771</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G29" s="11">
-        <v>21.550684931506851</v>
-      </c>
-      <c r="H29" s="11">
-        <v>55.021000000000001</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B30" s="9">
-        <v>2019</v>
-      </c>
-      <c r="C30" s="10">
-        <v>43526</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="G30" s="9">
-        <v>28.86849315068493</v>
-      </c>
-      <c r="H30" s="9">
-        <v>53.996000000000002</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A31" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B31" s="11">
-        <v>2019</v>
-      </c>
-      <c r="C31" s="12">
-        <v>43491</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="F31" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="G31" s="11">
-        <v>21.863013698630141</v>
-      </c>
-      <c r="H31" s="11">
-        <v>56.115000000000002</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B32" s="9">
-        <v>2019</v>
-      </c>
-      <c r="C32" s="10">
-        <v>43485</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="G32" s="9">
-        <v>30.843835616438351</v>
-      </c>
-      <c r="H32" s="9">
-        <v>51.448</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A33" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B33" s="11">
-        <v>2018</v>
-      </c>
-      <c r="C33" s="12">
-        <v>43450</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>189</v>
-      </c>
-      <c r="F33" s="11" t="s">
-        <v>190</v>
-      </c>
-      <c r="G33" s="11">
-        <v>30.74794520547945</v>
-      </c>
-      <c r="H33" s="11">
-        <v>51.945</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A34" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B34" s="9">
-        <v>2018</v>
-      </c>
-      <c r="C34" s="10">
-        <v>43436</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="G34" s="9">
-        <v>24.301369863013701</v>
-      </c>
-      <c r="H34" s="9">
-        <v>52.691000000000003</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A35" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35" s="11">
-        <v>2018</v>
-      </c>
-      <c r="C35" s="12">
-        <v>43398</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E35" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="F35" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11">
-        <v>53.145000000000003</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A36" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B36" s="9">
-        <v>2018</v>
-      </c>
-      <c r="C36" s="10">
-        <v>43393</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9">
-        <v>53.503</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A37" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B37" s="11">
-        <v>2018</v>
-      </c>
-      <c r="C37" s="12">
-        <v>43162</v>
-      </c>
-      <c r="D37" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>191</v>
-      </c>
-      <c r="F37" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11">
-        <v>52.222000000000001</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A38" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="B38" s="9">
-        <v>2018</v>
-      </c>
-      <c r="C38" s="10">
-        <v>43119</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E38" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9">
-        <v>53.103000000000002</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A39" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B39" s="11">
-        <v>2017</v>
-      </c>
-      <c r="C39" s="12">
-        <v>43077</v>
-      </c>
-      <c r="D39" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E39" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="F39" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11">
-        <v>53.011000000000003</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A40" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B40" s="9">
-        <v>2017</v>
-      </c>
-      <c r="C40" s="10">
-        <v>43070</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9">
-        <v>51.798000000000002</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A41" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B41" s="11">
-        <v>2017</v>
-      </c>
-      <c r="C41" s="12">
-        <v>43049</v>
-      </c>
-      <c r="D41" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E41" s="11" t="s">
-        <v>189</v>
-      </c>
-      <c r="F41" s="11" t="s">
-        <v>190</v>
-      </c>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11">
-        <v>54.125999999999998</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A42" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B42" s="9">
-        <v>2017</v>
-      </c>
-      <c r="C42" s="10">
-        <v>43042</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="G42" s="9"/>
-      <c r="H42" s="9">
-        <v>53.268999999999998</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A43" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B43" s="11">
-        <v>2017</v>
-      </c>
-      <c r="C43" s="12">
-        <v>42867</v>
-      </c>
-      <c r="D43" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="F43" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11">
-        <v>55.48</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A44" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B44" s="9">
-        <v>2017</v>
-      </c>
-      <c r="C44" s="10">
-        <v>42790</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="G44" s="9"/>
-      <c r="H44" s="9">
-        <v>51.09</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B45" s="11">
-        <v>2017</v>
-      </c>
-      <c r="C45" s="12">
-        <v>42783</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E45" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="F45" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="G45" s="11"/>
-      <c r="H45" s="11">
-        <v>56.390999999999998</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L133"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -21501,7 +20345,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="23" t="s">
         <v>25</v>
       </c>
@@ -21539,7 +20383,7 @@
         <v>56.962000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="23" t="s">
         <v>25</v>
       </c>
@@ -21577,7 +20421,7 @@
         <v>56.962000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="23" t="s">
         <v>25</v>
       </c>
@@ -21615,7 +20459,7 @@
         <v>56.962000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="25" t="s">
         <v>27</v>
       </c>
@@ -21653,7 +20497,7 @@
         <v>61.537999999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
         <v>27</v>
       </c>
@@ -21691,7 +20535,7 @@
         <v>61.537999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="25" t="s">
         <v>27</v>
       </c>
@@ -21843,7 +20687,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="25" t="s">
         <v>30</v>
       </c>
@@ -21881,7 +20725,7 @@
         <v>58.536585365853668</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="25" t="s">
         <v>30</v>
       </c>
@@ -21919,7 +20763,7 @@
         <v>58.536585365853668</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="25" t="s">
         <v>30</v>
       </c>
@@ -22071,7 +20915,7 @@
         <v>58.158000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="25" t="s">
         <v>32</v>
       </c>
@@ -22109,7 +20953,7 @@
         <v>55.988</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="25" t="s">
         <v>32</v>
       </c>
@@ -22147,7 +20991,7 @@
         <v>55.988</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="25" t="s">
         <v>32</v>
       </c>
@@ -22185,7 +21029,7 @@
         <v>55.988</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="23" t="s">
         <v>34</v>
       </c>
@@ -22223,7 +21067,7 @@
         <v>52.786000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="23" t="s">
         <v>34</v>
       </c>
@@ -22261,7 +21105,7 @@
         <v>52.786000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="23" t="s">
         <v>34</v>
       </c>
@@ -22299,7 +21143,7 @@
         <v>52.786000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="25" t="s">
         <v>27</v>
       </c>
@@ -22337,7 +21181,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="25" t="s">
         <v>27</v>
       </c>
@@ -22375,7 +21219,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="25" t="s">
         <v>27</v>
       </c>
@@ -22413,7 +21257,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="23" t="s">
         <v>35</v>
       </c>
@@ -22451,7 +21295,7 @@
         <v>53.811999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="23" t="s">
         <v>35</v>
       </c>
@@ -22489,7 +21333,7 @@
         <v>53.811999999999998</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="23" t="s">
         <v>35</v>
       </c>
@@ -22641,7 +21485,7 @@
         <v>56.515000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="23" t="s">
         <v>34</v>
       </c>
@@ -22679,7 +21523,7 @@
         <v>57.234000000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="23" t="s">
         <v>34</v>
       </c>
@@ -22717,7 +21561,7 @@
         <v>57.234000000000002</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>34</v>
       </c>
@@ -22755,7 +21599,7 @@
         <v>57.234000000000002</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="25" t="s">
         <v>37</v>
       </c>
@@ -22793,7 +21637,7 @@
         <v>53.651000000000003</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="25" t="s">
         <v>37</v>
       </c>
@@ -22831,7 +21675,7 @@
         <v>53.651000000000003</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="25" t="s">
         <v>37</v>
       </c>
@@ -22869,7 +21713,7 @@
         <v>53.651000000000003</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="23" t="s">
         <v>38</v>
       </c>
@@ -22907,7 +21751,7 @@
         <v>38.256999999999998</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="23" t="s">
         <v>38</v>
       </c>
@@ -22945,7 +21789,7 @@
         <v>38.256999999999998</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="23" t="s">
         <v>38</v>
       </c>
@@ -23091,7 +21935,7 @@
       </c>
       <c r="L43" s="25"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="23" t="s">
         <v>39</v>
       </c>
@@ -23129,7 +21973,7 @@
         <v>52.709000000000003</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="23" t="s">
         <v>39</v>
       </c>
@@ -23167,7 +22011,7 @@
         <v>52.709000000000003</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="23" t="s">
         <v>39</v>
       </c>
@@ -23205,7 +22049,7 @@
         <v>52.709000000000003</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>34</v>
       </c>
@@ -23243,7 +22087,7 @@
         <v>57.784999999999997</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="25" t="s">
         <v>34</v>
       </c>
@@ -23281,7 +22125,7 @@
         <v>57.784999999999997</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="25" t="s">
         <v>34</v>
       </c>
@@ -23319,7 +22163,7 @@
         <v>57.784999999999997</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="23" t="s">
         <v>36</v>
       </c>
@@ -23357,7 +22201,7 @@
         <v>56.161999999999999</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="23" t="s">
         <v>36</v>
       </c>
@@ -23395,7 +22239,7 @@
         <v>56.161999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="23" t="s">
         <v>36</v>
       </c>
@@ -23547,7 +22391,7 @@
         <v>57.052</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="23" t="s">
         <v>39</v>
       </c>
@@ -23585,7 +22429,7 @@
         <v>53.695999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="23" t="s">
         <v>39</v>
       </c>
@@ -23623,7 +22467,7 @@
         <v>53.695999999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="23" t="s">
         <v>39</v>
       </c>
@@ -23661,7 +22505,7 @@
         <v>53.695999999999998</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="25" t="s">
         <v>41</v>
       </c>
@@ -23699,7 +22543,7 @@
         <v>56.927999999999997</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="25" t="s">
         <v>41</v>
       </c>
@@ -23737,7 +22581,7 @@
         <v>56.927999999999997</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="25" t="s">
         <v>41</v>
       </c>
@@ -23775,7 +22619,7 @@
         <v>56.927999999999997</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="23" t="s">
         <v>42</v>
       </c>
@@ -23813,7 +22657,7 @@
         <v>54.893999999999998</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="23" t="s">
         <v>42</v>
       </c>
@@ -23851,7 +22695,7 @@
         <v>54.893999999999998</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="23" t="s">
         <v>42</v>
       </c>
@@ -24003,7 +22847,7 @@
         <v>57.43</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="23" t="s">
         <v>34</v>
       </c>
@@ -24041,7 +22885,7 @@
         <v>53.741</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="23" t="s">
         <v>34</v>
       </c>
@@ -24079,7 +22923,7 @@
         <v>53.741</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="23" t="s">
         <v>34</v>
       </c>
@@ -24117,7 +22961,7 @@
         <v>53.741</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="25" t="s">
         <v>44</v>
       </c>
@@ -24155,7 +22999,7 @@
         <v>54.131999999999998</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="25" t="s">
         <v>44</v>
       </c>
@@ -24193,7 +23037,7 @@
         <v>54.131999999999998</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="25" t="s">
         <v>44</v>
       </c>
@@ -24231,7 +23075,7 @@
         <v>54.131999999999998</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="23" t="s">
         <v>45</v>
       </c>
@@ -24269,7 +23113,7 @@
         <v>55.6</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="23" t="s">
         <v>45</v>
       </c>
@@ -24307,7 +23151,7 @@
         <v>55.6</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="23" t="s">
         <v>45</v>
       </c>
@@ -24345,7 +23189,7 @@
         <v>55.6</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="25" t="s">
         <v>27</v>
       </c>
@@ -24383,7 +23227,7 @@
         <v>56.533000000000001</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="25" t="s">
         <v>27</v>
       </c>
@@ -24421,7 +23265,7 @@
         <v>56.533000000000001</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="25" t="s">
         <v>27</v>
       </c>
@@ -24459,7 +23303,7 @@
         <v>56.533000000000001</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="23" t="s">
         <v>36</v>
       </c>
@@ -24497,7 +23341,7 @@
         <v>56.436</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="23" t="s">
         <v>36</v>
       </c>
@@ -24535,7 +23379,7 @@
         <v>56.436</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="23" t="s">
         <v>36</v>
       </c>
@@ -24573,7 +23417,7 @@
         <v>56.436</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="25" t="s">
         <v>46</v>
       </c>
@@ -24611,7 +23455,7 @@
         <v>56.390999999999998</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="25" t="s">
         <v>46</v>
       </c>
@@ -24649,7 +23493,7 @@
         <v>56.390999999999998</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="25" t="s">
         <v>46</v>
       </c>
@@ -24801,7 +23645,7 @@
         <v>56.91</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="25" t="s">
         <v>27</v>
       </c>
@@ -24839,7 +23683,7 @@
         <v>58.8</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="25" t="s">
         <v>27</v>
       </c>
@@ -24877,7 +23721,7 @@
         <v>58.8</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="25" t="s">
         <v>27</v>
       </c>
@@ -24915,7 +23759,7 @@
         <v>58.8</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="23" t="s">
         <v>45</v>
       </c>
@@ -24953,7 +23797,7 @@
         <v>55.996000000000002</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="23" t="s">
         <v>45</v>
       </c>
@@ -24991,7 +23835,7 @@
         <v>55.996000000000002</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="23" t="s">
         <v>45</v>
       </c>
@@ -25029,7 +23873,7 @@
         <v>55.996000000000002</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="25" t="s">
         <v>49</v>
       </c>
@@ -25067,7 +23911,7 @@
         <v>56.902000000000001</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="25" t="s">
         <v>49</v>
       </c>
@@ -25105,7 +23949,7 @@
         <v>56.902000000000001</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="25" t="s">
         <v>49</v>
       </c>
@@ -25143,7 +23987,7 @@
         <v>56.902000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="23" t="s">
         <v>43</v>
       </c>
@@ -25181,7 +24025,7 @@
         <v>55.228000000000002</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="23" t="s">
         <v>43</v>
       </c>
@@ -25219,7 +24063,7 @@
         <v>55.228000000000002</v>
       </c>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="23" t="s">
         <v>43</v>
       </c>
@@ -25257,7 +24101,7 @@
         <v>55.228000000000002</v>
       </c>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="25" t="s">
         <v>34</v>
       </c>
@@ -25293,7 +24137,7 @@
         <v>56.639000000000003</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="25" t="s">
         <v>34</v>
       </c>
@@ -25329,7 +24173,7 @@
         <v>56.639000000000003</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="25" t="s">
         <v>34</v>
       </c>
@@ -25365,7 +24209,7 @@
         <v>56.639000000000003</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="23" t="s">
         <v>32</v>
       </c>
@@ -25401,7 +24245,7 @@
         <v>54.497999999999998</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="23" t="s">
         <v>32</v>
       </c>
@@ -25437,7 +24281,7 @@
         <v>54.497999999999998</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="23" t="s">
         <v>32</v>
       </c>
@@ -25473,7 +24317,7 @@
         <v>54.497999999999998</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="25" t="s">
         <v>48</v>
       </c>
@@ -25509,7 +24353,7 @@
         <v>43.445999999999998</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="25" t="s">
         <v>48</v>
       </c>
@@ -25545,7 +24389,7 @@
         <v>43.445999999999998</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="25" t="s">
         <v>48</v>
       </c>
@@ -25581,7 +24425,7 @@
         <v>43.445999999999998</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="23" t="s">
         <v>46</v>
       </c>
@@ -25617,7 +24461,7 @@
         <v>53.319000000000003</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="23" t="s">
         <v>46</v>
       </c>
@@ -25653,7 +24497,7 @@
         <v>53.319000000000003</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="23" t="s">
         <v>46</v>
       </c>
@@ -25689,7 +24533,7 @@
         <v>53.319000000000003</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="25" t="s">
         <v>28</v>
       </c>
@@ -25725,7 +24569,7 @@
         <v>52.246000000000002</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="25" t="s">
         <v>28</v>
       </c>
@@ -25761,7 +24605,7 @@
         <v>52.246000000000002</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="25" t="s">
         <v>28</v>
       </c>
@@ -25797,7 +24641,7 @@
         <v>52.246000000000002</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="23" t="s">
         <v>34</v>
       </c>
@@ -25833,7 +24677,7 @@
         <v>54.948</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="23" t="s">
         <v>34</v>
       </c>
@@ -25869,7 +24713,7 @@
         <v>54.948</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="23" t="s">
         <v>34</v>
       </c>
@@ -25905,7 +24749,7 @@
         <v>54.948</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="25" t="s">
         <v>52</v>
       </c>
@@ -25941,7 +24785,7 @@
         <v>54.533000000000001</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="25" t="s">
         <v>52</v>
       </c>
@@ -25977,7 +24821,7 @@
         <v>54.533000000000001</v>
       </c>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="25" t="s">
         <v>52</v>
       </c>
@@ -26013,7 +24857,7 @@
         <v>54.533000000000001</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="23" t="s">
         <v>47</v>
       </c>
@@ -26049,7 +24893,7 @@
         <v>53.738999999999997</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="23" t="s">
         <v>47</v>
       </c>
@@ -26085,7 +24929,7 @@
         <v>53.738999999999997</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="23" t="s">
         <v>47</v>
       </c>
@@ -26229,7 +25073,7 @@
         <v>54.98</v>
       </c>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="23" t="s">
         <v>56</v>
       </c>
@@ -26265,7 +25109,7 @@
         <v>52.53</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="23" t="s">
         <v>56</v>
       </c>
@@ -26301,7 +25145,7 @@
         <v>52.53</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="23" t="s">
         <v>56</v>
       </c>
@@ -26337,7 +25181,7 @@
         <v>52.53</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="25" t="s">
         <v>39</v>
       </c>
@@ -26373,7 +25217,7 @@
         <v>52.033999999999999</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="25" t="s">
         <v>39</v>
       </c>
@@ -26409,7 +25253,7 @@
         <v>52.033999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="25" t="s">
         <v>39</v>
       </c>
@@ -26446,7 +25290,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:L133" xr:uid="{00000000-0009-0000-0000-000006000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="WCH"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="G101:G133">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>$E101="R1"</formula>
@@ -26458,6 +25308,1163 @@
       <formula>$E101="Q"</formula>
     </cfRule>
   </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:H45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.1796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="9">
+        <v>2026</v>
+      </c>
+      <c r="C2" s="10">
+        <v>46136</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G2" s="9">
+        <v>25.62191780821918</v>
+      </c>
+      <c r="H2" s="9">
+        <v>55.640999999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="11">
+        <v>2026</v>
+      </c>
+      <c r="C3" s="12">
+        <v>46129</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G3" s="11">
+        <v>23.55890410958904</v>
+      </c>
+      <c r="H3" s="11">
+        <v>56.962000000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="9">
+        <v>2025</v>
+      </c>
+      <c r="C4" s="10">
+        <v>45952</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="G4" s="9">
+        <v>36.402739726027399</v>
+      </c>
+      <c r="H4" s="9">
+        <v>57.143000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="11">
+        <v>2025</v>
+      </c>
+      <c r="C5" s="12">
+        <v>45730</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="G5" s="11">
+        <v>23.80821917808219</v>
+      </c>
+      <c r="H5" s="11">
+        <v>54.381</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="9">
+        <v>2024</v>
+      </c>
+      <c r="C6" s="10">
+        <v>45584</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G6" s="9">
+        <v>24.109589041095891</v>
+      </c>
+      <c r="H6" s="9">
+        <v>56.515000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="11">
+        <v>2024</v>
+      </c>
+      <c r="C7" s="12">
+        <v>45512</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G7" s="11">
+        <v>28.92602739726027</v>
+      </c>
+      <c r="H7" s="11">
+        <v>58.442</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="9">
+        <v>2024</v>
+      </c>
+      <c r="C8" s="10">
+        <v>45395</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="G8" s="9">
+        <v>37.536986301369858</v>
+      </c>
+      <c r="H8" s="9">
+        <v>56.25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="11">
+        <v>2024</v>
+      </c>
+      <c r="C9" s="12">
+        <v>45368</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G9" s="11">
+        <v>21.473972602739721</v>
+      </c>
+      <c r="H9" s="11">
+        <v>55.728000000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="9">
+        <v>2024</v>
+      </c>
+      <c r="C10" s="10">
+        <v>45325</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="G10" s="9">
+        <v>35.010958904109593</v>
+      </c>
+      <c r="H10" s="9">
+        <v>53.892000000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="11">
+        <v>2023</v>
+      </c>
+      <c r="C11" s="12">
+        <v>45144</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G11" s="11">
+        <v>25.109589041095891</v>
+      </c>
+      <c r="H11" s="11">
+        <v>54.795000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="9">
+        <v>2023</v>
+      </c>
+      <c r="C12" s="10">
+        <v>45038</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="G12" s="9">
+        <v>24.232876712328771</v>
+      </c>
+      <c r="H12" s="9">
+        <v>55.901000000000003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="11">
+        <v>2023</v>
+      </c>
+      <c r="C13" s="12">
+        <v>45001</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G13" s="11">
+        <v>29.07397260273973</v>
+      </c>
+      <c r="H13" s="11">
+        <v>53.097000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="9">
+        <v>2023</v>
+      </c>
+      <c r="C14" s="10">
+        <v>44982</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G14" s="9">
+        <v>27.761643835616439</v>
+      </c>
+      <c r="H14" s="9">
+        <v>52.173999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A15" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="11">
+        <v>2022</v>
+      </c>
+      <c r="C15" s="12">
+        <v>44849</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="11">
+        <v>31.906849315068492</v>
+      </c>
+      <c r="H15" s="11"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="9">
+        <v>2022</v>
+      </c>
+      <c r="C16" s="10">
+        <v>44752</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="G16" s="9">
+        <v>28.465753424657539</v>
+      </c>
+      <c r="H16" s="9">
+        <v>52.631999999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="11">
+        <v>2022</v>
+      </c>
+      <c r="C17" s="12">
+        <v>44696</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="11">
+        <v>23.671232876712331</v>
+      </c>
+      <c r="H17" s="11">
+        <v>53.097000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="9">
+        <v>2022</v>
+      </c>
+      <c r="C18" s="10">
+        <v>44675</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="G18" s="9">
+        <v>26.42739726027397</v>
+      </c>
+      <c r="H18" s="9">
+        <v>54.545000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="11">
+        <v>2021</v>
+      </c>
+      <c r="C19" s="12">
+        <v>44492</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G19" s="11">
+        <v>23.112328767123291</v>
+      </c>
+      <c r="H19" s="11">
+        <v>55.47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="9">
+        <v>2021</v>
+      </c>
+      <c r="C20" s="10">
+        <v>44451</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="G20" s="9">
+        <v>30.668493150684931</v>
+      </c>
+      <c r="H20" s="9">
+        <v>51.551000000000002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A21" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="11">
+        <v>2021</v>
+      </c>
+      <c r="C21" s="12">
+        <v>44413</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" s="11">
+        <v>23.30958904109589</v>
+      </c>
+      <c r="H21" s="11">
+        <v>56.539000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="9">
+        <v>2021</v>
+      </c>
+      <c r="C22" s="10">
+        <v>44388</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="9">
+        <v>23.038356164383561</v>
+      </c>
+      <c r="H22" s="9">
+        <v>53.85</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A23" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="11">
+        <v>2020</v>
+      </c>
+      <c r="C23" s="12">
+        <v>43890</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="G23" s="11">
+        <v>24.482191780821921</v>
+      </c>
+      <c r="H23" s="11"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="9">
+        <v>2020</v>
+      </c>
+      <c r="C24" s="10">
+        <v>43855</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="G24" s="9">
+        <v>25.164383561643831</v>
+      </c>
+      <c r="H24" s="9">
+        <v>53.784999999999997</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="11">
+        <v>2019</v>
+      </c>
+      <c r="C25" s="12">
+        <v>43813</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="G25" s="11">
+        <v>26.013698630136989</v>
+      </c>
+      <c r="H25" s="11">
+        <v>53.875</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="9">
+        <v>2019</v>
+      </c>
+      <c r="C26" s="10">
+        <v>43806</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="G26" s="9">
+        <v>25.030136986301368</v>
+      </c>
+      <c r="H26" s="9">
+        <v>54.192999999999998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="11">
+        <v>2019</v>
+      </c>
+      <c r="C27" s="12">
+        <v>43799</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="G27" s="11">
+        <v>31.8</v>
+      </c>
+      <c r="H27" s="11">
+        <v>53.749000000000002</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" s="9">
+        <v>2019</v>
+      </c>
+      <c r="C28" s="10">
+        <v>43779</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="G28" s="9">
+        <v>23.82465753424658</v>
+      </c>
+      <c r="H28" s="9"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B29" s="11">
+        <v>2019</v>
+      </c>
+      <c r="C29" s="12">
+        <v>43771</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G29" s="11">
+        <v>21.550684931506851</v>
+      </c>
+      <c r="H29" s="11">
+        <v>55.021000000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B30" s="9">
+        <v>2019</v>
+      </c>
+      <c r="C30" s="10">
+        <v>43526</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="G30" s="9">
+        <v>28.86849315068493</v>
+      </c>
+      <c r="H30" s="9">
+        <v>53.996000000000002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B31" s="11">
+        <v>2019</v>
+      </c>
+      <c r="C31" s="12">
+        <v>43491</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="G31" s="11">
+        <v>21.863013698630141</v>
+      </c>
+      <c r="H31" s="11">
+        <v>56.115000000000002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B32" s="9">
+        <v>2019</v>
+      </c>
+      <c r="C32" s="10">
+        <v>43485</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="G32" s="9">
+        <v>30.843835616438351</v>
+      </c>
+      <c r="H32" s="9">
+        <v>51.448</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B33" s="11">
+        <v>2018</v>
+      </c>
+      <c r="C33" s="12">
+        <v>43450</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="G33" s="11">
+        <v>30.74794520547945</v>
+      </c>
+      <c r="H33" s="11">
+        <v>51.945</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" s="9">
+        <v>2018</v>
+      </c>
+      <c r="C34" s="10">
+        <v>43436</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G34" s="9">
+        <v>24.301369863013701</v>
+      </c>
+      <c r="H34" s="9">
+        <v>52.691000000000003</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="11">
+        <v>2018</v>
+      </c>
+      <c r="C35" s="12">
+        <v>43398</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11">
+        <v>53.145000000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" s="9">
+        <v>2018</v>
+      </c>
+      <c r="C36" s="10">
+        <v>43393</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9">
+        <v>53.503</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A37" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B37" s="11">
+        <v>2018</v>
+      </c>
+      <c r="C37" s="12">
+        <v>43162</v>
+      </c>
+      <c r="D37" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E37" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="F37" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11">
+        <v>52.222000000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A38" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="9">
+        <v>2018</v>
+      </c>
+      <c r="C38" s="10">
+        <v>43119</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9">
+        <v>53.103000000000002</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A39" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B39" s="11">
+        <v>2017</v>
+      </c>
+      <c r="C39" s="12">
+        <v>43077</v>
+      </c>
+      <c r="D39" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E39" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="G39" s="11"/>
+      <c r="H39" s="11">
+        <v>53.011000000000003</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A40" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" s="9">
+        <v>2017</v>
+      </c>
+      <c r="C40" s="10">
+        <v>43070</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9">
+        <v>51.798000000000002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A41" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="11">
+        <v>2017</v>
+      </c>
+      <c r="C41" s="12">
+        <v>43049</v>
+      </c>
+      <c r="D41" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E41" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11">
+        <v>54.125999999999998</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A42" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42" s="9">
+        <v>2017</v>
+      </c>
+      <c r="C42" s="10">
+        <v>43042</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9">
+        <v>53.268999999999998</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A43" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B43" s="11">
+        <v>2017</v>
+      </c>
+      <c r="C43" s="12">
+        <v>42867</v>
+      </c>
+      <c r="D43" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="F43" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="G43" s="11"/>
+      <c r="H43" s="11">
+        <v>55.48</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A44" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B44" s="9">
+        <v>2017</v>
+      </c>
+      <c r="C44" s="10">
+        <v>42790</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9">
+        <v>51.09</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A45" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B45" s="11">
+        <v>2017</v>
+      </c>
+      <c r="C45" s="12">
+        <v>42783</v>
+      </c>
+      <c r="D45" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E45" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="F45" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="G45" s="11"/>
+      <c r="H45" s="11">
+        <v>56.390999999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -27629,6 +27636,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:R133"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -27695,7 +27703,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>25</v>
       </c>
@@ -27751,7 +27759,7 @@
         <v>55.215000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>25</v>
       </c>
@@ -27807,7 +27815,7 @@
         <v>55.215000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>25</v>
       </c>
@@ -27863,7 +27871,7 @@
         <v>55.215000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>27</v>
       </c>
@@ -27919,7 +27927,7 @@
         <v>58.442</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>27</v>
       </c>
@@ -27975,7 +27983,7 @@
         <v>58.442</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -28199,7 +28207,7 @@
         <v>56.356000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
         <v>30</v>
       </c>
@@ -28255,7 +28263,7 @@
         <v>56.284999999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
         <v>30</v>
       </c>
@@ -28311,7 +28319,7 @@
         <v>56.284999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>30</v>
       </c>
@@ -28535,7 +28543,7 @@
         <v>54.710999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="11" t="s">
         <v>32</v>
       </c>
@@ -28591,7 +28599,7 @@
         <v>55.728000000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
         <v>32</v>
       </c>
@@ -28647,7 +28655,7 @@
         <v>55.728000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="11" t="s">
         <v>32</v>
       </c>
@@ -28703,7 +28711,7 @@
         <v>55.728000000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>34</v>
       </c>
@@ -28759,7 +28767,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>34</v>
       </c>
@@ -28815,7 +28823,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
         <v>34</v>
       </c>
@@ -28871,7 +28879,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="11" t="s">
         <v>27</v>
       </c>
@@ -28927,7 +28935,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="11" t="s">
         <v>27</v>
       </c>
@@ -28983,7 +28991,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11" t="s">
         <v>27</v>
       </c>
@@ -29039,7 +29047,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="9" t="s">
         <v>35</v>
       </c>
@@ -29095,7 +29103,7 @@
         <v>51.195</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="s">
         <v>35</v>
       </c>
@@ -29151,7 +29159,7 @@
         <v>51.195</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="s">
         <v>35</v>
       </c>
@@ -29375,7 +29383,7 @@
         <v>57.765999999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="9" t="s">
         <v>34</v>
       </c>
@@ -29431,7 +29439,7 @@
         <v>55.283000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="s">
         <v>34</v>
       </c>
@@ -29487,7 +29495,7 @@
         <v>55.283000000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="s">
         <v>34</v>
       </c>
@@ -29543,7 +29551,7 @@
         <v>55.283000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="11" t="s">
         <v>37</v>
       </c>
@@ -29599,7 +29607,7 @@
         <v>54.25</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="11" t="s">
         <v>37</v>
       </c>
@@ -29655,7 +29663,7 @@
         <v>54.25</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="11" t="s">
         <v>37</v>
       </c>
@@ -29711,7 +29719,7 @@
         <v>54.25</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="s">
         <v>38</v>
       </c>
@@ -29767,7 +29775,7 @@
         <v>53.411999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="s">
         <v>38</v>
       </c>
@@ -29823,7 +29831,7 @@
         <v>53.411999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="9" t="s">
         <v>38</v>
       </c>
@@ -30041,7 +30049,7 @@
       </c>
       <c r="R43" s="11"/>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="s">
         <v>39</v>
       </c>
@@ -30097,7 +30105,7 @@
         <v>52.052999999999997</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="s">
         <v>39</v>
       </c>
@@ -30153,7 +30161,7 @@
         <v>52.052999999999997</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
         <v>39</v>
       </c>
@@ -30209,7 +30217,7 @@
         <v>52.052999999999997</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
@@ -30265,7 +30273,7 @@
         <v>54.314999999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
@@ -30321,7 +30329,7 @@
         <v>54.314999999999998</v>
       </c>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
@@ -30377,7 +30385,7 @@
         <v>54.314999999999998</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
         <v>36</v>
       </c>
@@ -30433,7 +30441,7 @@
         <v>54.281999999999996</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
         <v>36</v>
       </c>
@@ -30489,7 +30497,7 @@
         <v>54.281999999999996</v>
       </c>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
         <v>36</v>
       </c>
@@ -30713,7 +30721,7 @@
         <v>54.216999999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="9" t="s">
         <v>39</v>
       </c>
@@ -30769,7 +30777,7 @@
         <v>50.137999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="s">
         <v>39</v>
       </c>
@@ -30825,7 +30833,7 @@
         <v>50.137999999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="9" t="s">
         <v>39</v>
       </c>
@@ -30881,7 +30889,7 @@
         <v>50.137999999999998</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="11" t="s">
         <v>41</v>
       </c>
@@ -30937,7 +30945,7 @@
         <v>55.107999999999997</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="11" t="s">
         <v>41</v>
       </c>
@@ -30993,7 +31001,7 @@
         <v>55.107999999999997</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="11" t="s">
         <v>41</v>
       </c>
@@ -31049,7 +31057,7 @@
         <v>55.107999999999997</v>
       </c>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="9" t="s">
         <v>42</v>
       </c>
@@ -31105,7 +31113,7 @@
         <v>51.48</v>
       </c>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="9" t="s">
         <v>42</v>
       </c>
@@ -31161,7 +31169,7 @@
         <v>51.48</v>
       </c>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="9" t="s">
         <v>42</v>
       </c>
@@ -31385,7 +31393,7 @@
         <v>54.576000000000001</v>
       </c>
     </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="9" t="s">
         <v>34</v>
       </c>
@@ -31441,7 +31449,7 @@
         <v>53.93</v>
       </c>
     </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="9" t="s">
         <v>34</v>
       </c>
@@ -31497,7 +31505,7 @@
         <v>53.93</v>
       </c>
     </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="9" t="s">
         <v>34</v>
       </c>
@@ -31553,7 +31561,7 @@
         <v>53.93</v>
       </c>
     </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="11" t="s">
         <v>44</v>
       </c>
@@ -31609,7 +31617,7 @@
         <v>53.168999999999997</v>
       </c>
     </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="11" t="s">
         <v>44</v>
       </c>
@@ -31665,7 +31673,7 @@
         <v>53.168999999999997</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="11" t="s">
         <v>44</v>
       </c>
@@ -31721,7 +31729,7 @@
         <v>53.168999999999997</v>
       </c>
     </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="9" t="s">
         <v>45</v>
       </c>
@@ -31777,7 +31785,7 @@
         <v>54.075000000000003</v>
       </c>
     </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="9" t="s">
         <v>45</v>
       </c>
@@ -31833,7 +31841,7 @@
         <v>54.075000000000003</v>
       </c>
     </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="9" t="s">
         <v>45</v>
       </c>
@@ -31889,7 +31897,7 @@
         <v>54.075000000000003</v>
       </c>
     </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="11" t="s">
         <v>27</v>
       </c>
@@ -31945,7 +31953,7 @@
         <v>55.494999999999997</v>
       </c>
     </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="11" t="s">
         <v>27</v>
       </c>
@@ -32001,7 +32009,7 @@
         <v>55.494999999999997</v>
       </c>
     </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="11" t="s">
         <v>27</v>
       </c>
@@ -32057,7 +32065,7 @@
         <v>55.494999999999997</v>
       </c>
     </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="9" t="s">
         <v>36</v>
       </c>
@@ -32113,7 +32121,7 @@
         <v>53.826000000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="9" t="s">
         <v>36</v>
       </c>
@@ -32169,7 +32177,7 @@
         <v>53.826000000000001</v>
       </c>
     </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="9" t="s">
         <v>36</v>
       </c>
@@ -32225,7 +32233,7 @@
         <v>53.826000000000001</v>
       </c>
     </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="11" t="s">
         <v>46</v>
       </c>
@@ -32281,7 +32289,7 @@
         <v>53.822000000000003</v>
       </c>
     </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="11" t="s">
         <v>46</v>
       </c>
@@ -32337,7 +32345,7 @@
         <v>53.822000000000003</v>
       </c>
     </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="11" t="s">
         <v>46</v>
       </c>
@@ -32561,7 +32569,7 @@
         <v>54.338000000000001</v>
       </c>
     </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="11" t="s">
         <v>27</v>
       </c>
@@ -32617,7 +32625,7 @@
         <v>54.046999999999997</v>
       </c>
     </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="11" t="s">
         <v>27</v>
       </c>
@@ -32673,7 +32681,7 @@
         <v>54.046999999999997</v>
       </c>
     </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="11" t="s">
         <v>27</v>
       </c>
@@ -32729,7 +32737,7 @@
         <v>54.046999999999997</v>
       </c>
     </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="9" t="s">
         <v>45</v>
       </c>
@@ -32785,7 +32793,7 @@
         <v>51.37</v>
       </c>
     </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="9" t="s">
         <v>45</v>
       </c>
@@ -32841,7 +32849,7 @@
         <v>51.37</v>
       </c>
     </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="9" t="s">
         <v>45</v>
       </c>
@@ -32897,7 +32905,7 @@
         <v>51.37</v>
       </c>
     </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="11" t="s">
         <v>49</v>
       </c>
@@ -32953,7 +32961,7 @@
         <v>52.722999999999999</v>
       </c>
     </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="11" t="s">
         <v>49</v>
       </c>
@@ -33009,7 +33017,7 @@
         <v>52.722999999999999</v>
       </c>
     </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="11" t="s">
         <v>49</v>
       </c>
@@ -33065,7 +33073,7 @@
         <v>52.722999999999999</v>
       </c>
     </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="9" t="s">
         <v>43</v>
       </c>
@@ -33121,7 +33129,7 @@
         <v>52.741999999999997</v>
       </c>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="9" t="s">
         <v>43</v>
       </c>
@@ -33177,7 +33185,7 @@
         <v>52.741999999999997</v>
       </c>
     </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="9" t="s">
         <v>43</v>
       </c>
@@ -33233,7 +33241,7 @@
         <v>52.741999999999997</v>
       </c>
     </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="11" t="s">
         <v>34</v>
       </c>
@@ -33287,7 +33295,7 @@
         <v>52.878999999999998</v>
       </c>
     </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="11" t="s">
         <v>34</v>
       </c>
@@ -33341,7 +33349,7 @@
         <v>52.878999999999998</v>
       </c>
     </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="11" t="s">
         <v>34</v>
       </c>
@@ -33395,7 +33403,7 @@
         <v>52.878999999999998</v>
       </c>
     </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="9" t="s">
         <v>32</v>
       </c>
@@ -33449,7 +33457,7 @@
         <v>53.993000000000002</v>
       </c>
     </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="9" t="s">
         <v>32</v>
       </c>
@@ -33503,7 +33511,7 @@
         <v>53.993000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="9" t="s">
         <v>32</v>
       </c>
@@ -33557,7 +33565,7 @@
         <v>53.993000000000002</v>
       </c>
     </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="11" t="s">
         <v>48</v>
       </c>
@@ -33611,7 +33619,7 @@
         <v>54.491</v>
       </c>
     </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="11" t="s">
         <v>48</v>
       </c>
@@ -33665,7 +33673,7 @@
         <v>54.491</v>
       </c>
     </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="11" t="s">
         <v>48</v>
       </c>
@@ -33719,7 +33727,7 @@
         <v>54.491</v>
       </c>
     </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="9" t="s">
         <v>46</v>
       </c>
@@ -33773,7 +33781,7 @@
         <v>51.802999999999997</v>
       </c>
     </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="9" t="s">
         <v>46</v>
       </c>
@@ -33827,7 +33835,7 @@
         <v>51.802999999999997</v>
       </c>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="9" t="s">
         <v>46</v>
       </c>
@@ -33881,7 +33889,7 @@
         <v>51.802999999999997</v>
       </c>
     </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="11" t="s">
         <v>28</v>
       </c>
@@ -33935,7 +33943,7 @@
         <v>51.274000000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="11" t="s">
         <v>28</v>
       </c>
@@ -33989,7 +33997,7 @@
         <v>51.274000000000001</v>
       </c>
     </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="11" t="s">
         <v>28</v>
       </c>
@@ -34043,7 +34051,7 @@
         <v>51.274000000000001</v>
       </c>
     </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="9" t="s">
         <v>34</v>
       </c>
@@ -34097,7 +34105,7 @@
         <v>52.695999999999998</v>
       </c>
     </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="9" t="s">
         <v>34</v>
       </c>
@@ -34151,7 +34159,7 @@
         <v>52.695999999999998</v>
       </c>
     </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="9" t="s">
         <v>34</v>
       </c>
@@ -34205,7 +34213,7 @@
         <v>52.695999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="11" t="s">
         <v>52</v>
       </c>
@@ -34259,7 +34267,7 @@
         <v>54.171999999999997</v>
       </c>
     </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="11" t="s">
         <v>52</v>
       </c>
@@ -34313,7 +34321,7 @@
         <v>54.171999999999997</v>
       </c>
     </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="11" t="s">
         <v>52</v>
       </c>
@@ -34367,7 +34375,7 @@
         <v>54.171999999999997</v>
       </c>
     </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="9" t="s">
         <v>47</v>
       </c>
@@ -34421,7 +34429,7 @@
         <v>52.085000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="9" t="s">
         <v>47</v>
       </c>
@@ -34475,7 +34483,7 @@
         <v>52.085000000000001</v>
       </c>
     </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="9" t="s">
         <v>47</v>
       </c>
@@ -34691,7 +34699,7 @@
         <v>52.703000000000003</v>
       </c>
     </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="9" t="s">
         <v>56</v>
       </c>
@@ -34745,7 +34753,7 @@
         <v>50.832999999999998</v>
       </c>
     </row>
-    <row r="129" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="9" t="s">
         <v>56</v>
       </c>
@@ -34799,7 +34807,7 @@
         <v>50.832999999999998</v>
       </c>
     </row>
-    <row r="130" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="9" t="s">
         <v>56</v>
       </c>
@@ -34853,7 +34861,7 @@
         <v>50.832999999999998</v>
       </c>
     </row>
-    <row r="131" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="11" t="s">
         <v>39</v>
       </c>
@@ -34907,7 +34915,7 @@
         <v>51.021999999999998</v>
       </c>
     </row>
-    <row r="132" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="11" t="s">
         <v>39</v>
       </c>
@@ -34961,7 +34969,7 @@
         <v>51.021999999999998</v>
       </c>
     </row>
-    <row r="133" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="11" t="s">
         <v>39</v>
       </c>
@@ -35016,7 +35024,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R1" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
+  <autoFilter ref="A1:R133" xr:uid="{00000000-0009-0000-0000-000008000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="WCH"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="I2:I133">
     <cfRule type="colorScale" priority="13">
       <colorScale>

</xml_diff>